<commit_message>
adding plot outputs for poster
</commit_message>
<xml_diff>
--- a/ARDUINO/prototype_REV1/plots/organic_waste_mar09.xlsx
+++ b/ARDUINO/prototype_REV1/plots/organic_waste_mar09.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Isaac\source\repos\F.R.E.D\ARDUINO\prototype_REV1\plots\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E738FAA1-E245-4C30-B289-9CB1575745CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E62D394D-8D12-44A3-B83F-1344EC9B412A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2C441D20-A01D-45BC-BB19-2A07FE850A91}"/>
   </bookViews>
@@ -211,7 +211,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-CA"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -9820,7 +9820,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000009-B255-4FF0-B45F-1EADFBD17E27}"/>
                   </c:ext>
@@ -10796,7 +10796,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{0000000A-B255-4FF0-B45F-1EADFBD17E27}"/>
                   </c:ext>
@@ -11772,7 +11772,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{0000000B-B255-4FF0-B45F-1EADFBD17E27}"/>
                   </c:ext>
@@ -11845,7 +11845,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-CA"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -11917,7 +11917,7 @@
         <c:title>
           <c:tx>
             <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -11954,7 +11954,7 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
@@ -11970,7 +11970,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-CA"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -12038,7 +12038,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:ln w="3175">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
@@ -15108,7 +15108,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000001-A372-4918-A223-91B5984D948B}"/>
                   </c:ext>
@@ -16082,7 +16082,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000002-A372-4918-A223-91B5984D948B}"/>
                   </c:ext>
@@ -17053,7 +17053,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000003-A372-4918-A223-91B5984D948B}"/>
                   </c:ext>
@@ -18027,7 +18027,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000004-A372-4918-A223-91B5984D948B}"/>
                   </c:ext>
@@ -18998,7 +18998,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000005-A372-4918-A223-91B5984D948B}"/>
                   </c:ext>
@@ -19971,7 +19971,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000006-A372-4918-A223-91B5984D948B}"/>
                   </c:ext>
@@ -20944,7 +20944,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000007-A372-4918-A223-91B5984D948B}"/>
                   </c:ext>
@@ -21920,7 +21920,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000008-A372-4918-A223-91B5984D948B}"/>
                   </c:ext>
@@ -22896,7 +22896,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000009-A372-4918-A223-91B5984D948B}"/>
                   </c:ext>
@@ -23872,7 +23872,7 @@
                   </c:numRef>
                 </c:val>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{0000000A-A372-4918-A223-91B5984D948B}"/>
                   </c:ext>

</xml_diff>